<commit_message>
V2.4 atualização  tela 2, prog 2
</commit_message>
<xml_diff>
--- a/codigo/word_templates/FOLHA DE DADOS EQUIPAMENTO EXCEL.xlsx
+++ b/codigo/word_templates/FOLHA DE DADOS EQUIPAMENTO EXCEL.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc0c8436bbcd5584/Repositórios/app.esienergia/codigo/word_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{4BC2FFF5-BC24-4F7A-A0B0-4C3481730B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49363E46-9410-4DD1-96DE-546DD3B669A5}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{4BC2FFF5-BC24-4F7A-A0B0-4C3481730B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{356C5A89-80C5-43A3-9A3B-2F7D514F7093}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{4A893E87-B67C-414E-8C7E-76196958FBD9}"/>
   </bookViews>
   <sheets>
     <sheet name="FD EQUIP 1" sheetId="2" r:id="rId1"/>
-    <sheet name="Planilha1" sheetId="1" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
     <definedName name="Categoria">[1]Auxiliar!$K$2:$S$2</definedName>
@@ -71,10 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="57">
-  <si>
-    <t>FOLHA DE DADOS - Wall Mounted WM-01</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
   <si>
     <t>N° OC</t>
   </si>
@@ -241,7 +237,7 @@
     <t>OPCIONAIS</t>
   </si>
   <si>
-    <t>AUX</t>
+    <t xml:space="preserve">FOLHA DE DADOS - </t>
   </si>
 </sst>
 </file>
@@ -614,7 +610,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -685,27 +681,27 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -733,6 +729,42 @@
     <xf numFmtId="49" fontId="6" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -745,43 +777,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1119,6 +1114,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1502,7 +1501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DA14E58-E30C-4250-87CA-42591253E3B0}">
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.6640625" customWidth="1"/>
@@ -1511,132 +1510,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="47"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B2" s="49"/>
+      <c r="C2" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="51"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="40" t="s">
+      <c r="D2" s="53"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="55"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="48"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="43"/>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="40" t="s">
+      <c r="D3" s="53"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="55"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="48"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="43"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52"/>
-      <c r="B4" s="53"/>
-      <c r="C4" s="40" t="s">
+      <c r="D4" s="53"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="55"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="48"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="43"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="52"/>
-      <c r="B5" s="53"/>
-      <c r="C5" s="40" t="s">
+      <c r="D5" s="53"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="55"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="50"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="43"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54"/>
-      <c r="B6" s="55"/>
-      <c r="C6" s="40" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="41"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="43"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="55"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H7" s="44"/>
-      <c r="I7" s="45"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="41"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
       <c r="E8" s="5"/>
       <c r="F8" s="6"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="48"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="44"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="37" t="s">
         <v>13</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>14</v>
       </c>
       <c r="C9" s="38"/>
       <c r="D9" s="39"/>
       <c r="E9" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="21"/>
@@ -1645,15 +1644,15 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="37" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>17</v>
       </c>
       <c r="C10" s="38"/>
       <c r="D10" s="39"/>
       <c r="E10" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="21"/>
@@ -1662,15 +1661,15 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="30" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>19</v>
       </c>
       <c r="C11" s="19"/>
       <c r="D11" s="20"/>
       <c r="E11" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="21"/>
@@ -1679,15 +1678,15 @@
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="30" t="s">
         <v>20</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>21</v>
       </c>
       <c r="C12" s="19"/>
       <c r="D12" s="20"/>
       <c r="E12" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="21"/>
@@ -1696,15 +1695,15 @@
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="30" t="s">
         <v>22</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="20"/>
       <c r="E13" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="21"/>
@@ -1713,10 +1712,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="31" t="s">
         <v>24</v>
-      </c>
-      <c r="B14" s="31" t="s">
-        <v>25</v>
       </c>
       <c r="C14" s="32"/>
       <c r="D14" s="33"/>
@@ -1728,15 +1727,15 @@
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="30" t="s">
         <v>26</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>27</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="20"/>
       <c r="E15" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="21"/>
@@ -1745,15 +1744,15 @@
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="30" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>29</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="20"/>
       <c r="E16" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="21"/>
@@ -1762,15 +1761,15 @@
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="30" t="s">
         <v>30</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>31</v>
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="20"/>
       <c r="E17" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="21"/>
@@ -1779,10 +1778,10 @@
     </row>
     <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="30" t="s">
         <v>32</v>
-      </c>
-      <c r="B18" s="24" t="s">
-        <v>33</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="20"/>
@@ -1794,10 +1793,10 @@
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="31" t="s">
         <v>34</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>35</v>
       </c>
       <c r="C19" s="32"/>
       <c r="D19" s="33"/>
@@ -1809,15 +1808,15 @@
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="30" t="s">
         <v>36</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>37</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="20"/>
       <c r="E20" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="21"/>
@@ -1826,15 +1825,15 @@
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="30" t="s">
         <v>38</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>39</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="20"/>
       <c r="E21" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="21"/>
@@ -1843,10 +1842,10 @@
     </row>
     <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="31" t="s">
         <v>40</v>
-      </c>
-      <c r="B22" s="31" t="s">
-        <v>41</v>
       </c>
       <c r="C22" s="32"/>
       <c r="D22" s="33"/>
@@ -1858,15 +1857,15 @@
     </row>
     <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="30" t="s">
         <v>42</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>43</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="20"/>
       <c r="E23" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="21"/>
@@ -1875,15 +1874,15 @@
     </row>
     <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="30" t="s">
         <v>44</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>45</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="20"/>
       <c r="E24" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="21"/>
@@ -1892,15 +1891,15 @@
     </row>
     <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="30" t="s">
         <v>46</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>47</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="20"/>
       <c r="E25" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="21"/>
@@ -1909,15 +1908,15 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="30" t="s">
         <v>48</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>49</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="20"/>
       <c r="E26" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="21"/>
@@ -1926,15 +1925,15 @@
     </row>
     <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="30" t="s">
         <v>50</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>51</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="20"/>
       <c r="E27" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="21"/>
@@ -1943,15 +1942,15 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="30" t="s">
         <v>52</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>53</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="20"/>
       <c r="E28" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="21"/>
@@ -1960,10 +1959,10 @@
     </row>
     <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="31" t="s">
         <v>54</v>
-      </c>
-      <c r="B29" s="31" t="s">
-        <v>55</v>
       </c>
       <c r="C29" s="32"/>
       <c r="D29" s="33"/>
@@ -1975,7 +1974,7 @@
     </row>
     <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
-      <c r="B30" s="24"/>
+      <c r="B30" s="30"/>
       <c r="C30" s="19"/>
       <c r="D30" s="20"/>
       <c r="E30" s="10"/>
@@ -1986,7 +1985,7 @@
     </row>
     <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7"/>
-      <c r="B31" s="24"/>
+      <c r="B31" s="30"/>
       <c r="C31" s="19"/>
       <c r="D31" s="20"/>
       <c r="E31" s="10"/>
@@ -1997,7 +1996,7 @@
     </row>
     <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7"/>
-      <c r="B32" s="24"/>
+      <c r="B32" s="30"/>
       <c r="C32" s="19"/>
       <c r="D32" s="20"/>
       <c r="E32" s="10"/>
@@ -2006,9 +2005,9 @@
       <c r="H32" s="22"/>
       <c r="I32" s="23"/>
     </row>
-    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7"/>
-      <c r="B33" s="24"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="19"/>
       <c r="D33" s="20"/>
       <c r="E33" s="10"/>
@@ -2017,9 +2016,9 @@
       <c r="H33" s="22"/>
       <c r="I33" s="23"/>
     </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7"/>
-      <c r="B34" s="24"/>
+      <c r="B34" s="30"/>
       <c r="C34" s="19"/>
       <c r="D34" s="20"/>
       <c r="E34" s="10"/>
@@ -2028,9 +2027,9 @@
       <c r="H34" s="22"/>
       <c r="I34" s="23"/>
     </row>
-    <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7"/>
-      <c r="B35" s="24"/>
+      <c r="B35" s="30"/>
       <c r="C35" s="19"/>
       <c r="D35" s="20"/>
       <c r="E35" s="10"/>
@@ -2039,9 +2038,9 @@
       <c r="H35" s="22"/>
       <c r="I35" s="23"/>
     </row>
-    <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7"/>
-      <c r="B36" s="24"/>
+      <c r="B36" s="30"/>
       <c r="C36" s="19"/>
       <c r="D36" s="20"/>
       <c r="E36" s="10"/>
@@ -2049,20 +2048,19 @@
       <c r="G36" s="21"/>
       <c r="H36" s="22"/>
       <c r="I36" s="23"/>
-      <c r="K36" s="56"/>
-    </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11"/>
-      <c r="B37" s="25"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="27"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26"/>
       <c r="E37" s="12"/>
       <c r="F37" s="13"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="30"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G37" s="27"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="14"/>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
@@ -2073,7 +2071,7 @@
       <c r="H38" s="22"/>
       <c r="I38" s="23"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="16"/>
       <c r="B39" s="19"/>
       <c r="C39" s="19"/>
@@ -2084,7 +2082,7 @@
       <c r="H39" s="22"/>
       <c r="I39" s="23"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="16"/>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
@@ -2095,7 +2093,7 @@
       <c r="H40" s="22"/>
       <c r="I40" s="23"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="16"/>
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
@@ -2106,17 +2104,11 @@
       <c r="H41" s="22"/>
       <c r="I41" s="23"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="17"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B44">
-        <f>IF(F10="Wall Mounted",1,IF(F10="Split System",2,IF(F10="Self Contained",3,0)))</f>
-        <v>0</v>
-      </c>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="82">
@@ -2192,16 +2184,16 @@
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="G36:I36"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="G41:I41"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="G37:I37"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="G38:I38"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="G39:I39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="G41:I41"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F17" xr:uid="{B97C85C9-E3A1-491A-B92C-35F8275B38C2}">
@@ -2224,13 +2216,4 @@
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.19685039370078741" footer="0.19685039370078741"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70F748CB-53F6-4A88-8629-B056A27492AB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>